<commit_message>
FINDING: N/A LANE: NON-FINANCIAL — LEAD 443.281: register update 7:45 PM CT (rows 87/91/92 DONE-LIVE from #27383; 89/90 443.283 rebased; new 200 A/R KPI tie-out, 201-202 main static reds)
Docs only: docs/bus/lead/LEAD-PENDING-REGISTER.xlsx + .md. Every status from a measured
exit code or live number; no code change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0112DqKNUusL2t72oep2o5Jj
</commit_message>
<xml_diff>
--- a/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
+++ b/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Register" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Register'!$A$2:$L$201</definedName>
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L201"/>
+  <dimension ref="A1:L204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -502,7 +502,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 6:35 PM CT · every item numbered · DONE only with live proof</t>
+          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 7:45 PM CT · every item numbered · DONE only with live proof</t>
         </is>
       </c>
     </row>
@@ -5282,12 +5282,12 @@
       </c>
       <c r="J89" s="9" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>DONE-LIVE</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
         <is>
-          <t>LEAD 443.282 758bd029: guard credits tables read through a read view (D074 cache); selftest lock</t>
+          <t>LEAD #27383 d85ade3b: guard credits view-read tables; verify-no-dead-schema exit 0 on main</t>
         </is>
       </c>
       <c r="L89" s="3" t="inlineStr">
@@ -5403,7 +5403,7 @@
       </c>
       <c r="K91" s="3" t="inlineStr">
         <is>
-          <t>LEAD 443.283: one source; Manual opens from authoritative cash when no saved opening</t>
+          <t>LEAD 443.283 ea892ec5 rebased onto #27390: Manual opens at authoritative $25,533.37; tests 3/3, fe+be tsc 0; push waits on main reds</t>
         </is>
       </c>
       <c r="L91" s="3" t="inlineStr">
@@ -5463,7 +5463,7 @@
       </c>
       <c r="K92" s="3" t="inlineStr">
         <is>
-          <t>LEAD 443.283 f03a33c4: /cash-flow/opening-cash = BofA $8,202.50 + Relay $17,330.87 = $25,533.37; tests 3/3; pushing</t>
+          <t>LEAD 443.283: bank list = operating accounts only (BofA Plaid + Relay ledger); card payables/Faro removed</t>
         </is>
       </c>
       <c r="L92" s="3" t="inlineStr">
@@ -5518,12 +5518,12 @@
       </c>
       <c r="J93" s="9" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>DONE-LIVE</t>
         </is>
       </c>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>LEAD 443.282 cc74c41e/082a09a6: actuals from operating bank (Oct $208,031.56 in / $205,270.54 out posted); pushing</t>
+          <t>LEAD #27383 d85ade3b live: AvP Oct actual income $208,031.56 / expense $205,270.54 from operating bank; 283b is_credit form (exit 0 direction guard)</t>
         </is>
       </c>
       <c r="L93" s="3" t="inlineStr">
@@ -5578,12 +5578,12 @@
       </c>
       <c r="J94" s="9" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>DONE-LIVE</t>
         </is>
       </c>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>LEAD 443.282: pointer matched_advance_id -&gt; matched_factoring_advance_id (25 advances $202,044.98); pushing</t>
+          <t>LEAD #27383: rolling ledger factoring advances matched by bt.matched_factoring_advance_id; no double count</t>
         </is>
       </c>
       <c r="L94" s="3" t="inlineStr">
@@ -11839,6 +11839,170 @@
           <t>10-24 02:00 UTC</t>
         </is>
       </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>F · Money tie-outs</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D202" s="3" t="inlineStr">
+        <is>
+          <t>Accounting "Open invoices" KPI $624,076.72/165 vs GL A/R 1100 $621,076.72/164</t>
+        </is>
+      </c>
+      <c r="E202" s="3" t="inlineStr">
+        <is>
+          <t>prod 7:22 PM: diff $3,000.00 = 1 proforma (169-13690)</t>
+        </is>
+      </c>
+      <c r="F202" s="3" t="inlineStr">
+        <is>
+          <t>KPI filtered only void; proforma counted</t>
+        </is>
+      </c>
+      <c r="G202" s="3" t="inlineStr">
+        <is>
+          <t>issuedInvoice predicate on all 4 KPI aggregates + guard test</t>
+        </is>
+      </c>
+      <c r="H202" s="3" t="inlineStr">
+        <is>
+          <t>LEAD</t>
+        </is>
+      </c>
+      <c r="I202" s="3" t="inlineStr">
+        <is>
+          <t>443.285</t>
+        </is>
+      </c>
+      <c r="J202" s="7" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K202" s="3" t="inlineStr">
+        <is>
+          <t>9ef89188 test 3/3, be tsc 0; push waits on main reds</t>
+        </is>
+      </c>
+      <c r="L202" s="3" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="3" t="n">
+        <v>201</v>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>E · Main static reds</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D203" s="3" t="inlineStr">
+        <is>
+          <t>443.284: 7 main static reds from 10-23 board merges block every push</t>
+        </is>
+      </c>
+      <c r="E203" s="3" t="inlineStr">
+        <is>
+          <t>7:40 PM measured: 2 fixed (parity footer, factoring nav), 5 red</t>
+        </is>
+      </c>
+      <c r="F203" s="3" t="inlineStr">
+        <is>
+          <t>board merges changed contracts guards pin</t>
+        </is>
+      </c>
+      <c r="G203" s="3" t="inlineStr">
+        <is>
+          <t>retarget guards to board contract with failing plants; never baseline</t>
+        </is>
+      </c>
+      <c r="H203" s="3" t="inlineStr">
+        <is>
+          <t>CC-2/CC-3</t>
+        </is>
+      </c>
+      <c r="I203" s="3" t="inlineStr">
+        <is>
+          <t>443.284</t>
+        </is>
+      </c>
+      <c r="J203" s="7" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K203" s="3" t="inlineStr">
+        <is>
+          <t>CC-2: dashboard-connectivity, sweep-pre-list, test-provider; CC-3: partial-optional-chain, unselected-boxes</t>
+        </is>
+      </c>
+      <c r="L203" s="3" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="n">
+        <v>202</v>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>E · Main static reds</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>Fuel</t>
+        </is>
+      </c>
+      <c r="D204" s="3" t="inlineStr">
+        <is>
+          <t>verify-no-internal-payload-in-notes red: dreamline-statement-import memo interpolates input.expenseId</t>
+        </is>
+      </c>
+      <c r="E204" s="3" t="inlineStr">
+        <is>
+          <t>exit 1 on main 1c118712</t>
+        </is>
+      </c>
+      <c r="F204" s="3" t="inlineStr">
+        <is>
+          <t>afd3fd334e memo template</t>
+        </is>
+      </c>
+      <c r="G204" s="3" t="inlineStr">
+        <is>
+          <t>human memo + spine link</t>
+        </is>
+      </c>
+      <c r="H204" s="3" t="inlineStr">
+        <is>
+          <t>CC-2</t>
+        </is>
+      </c>
+      <c r="I204" s="3" t="inlineStr">
+        <is>
+          <t>443.284</t>
+        </is>
+      </c>
+      <c r="J204" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K204" s="3" t="inlineStr"/>
+      <c r="L204" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:L201"/>

</xml_diff>

<commit_message>
FINDING: N/A LANE: NON-FINANCIAL — LEAD 443.288: owner ruling (every expense-to-load assignment confirmed by dispatcher or closer; child documents follow their receipt) + register rows 203-207
Docs only: docs/bus/lead/OWNER-RULING-443.288-EXPENSE-LOAD-CONFIRMED-BY-DISPATCH-OR-CLOSER.md (owner verbatim
10-23 7:59 PM CT, measured root cause, the rule, assignment) and docs/bus/lead/LEAD-PENDING-REGISTER.xlsx/.md.
No code change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0112DqKNUusL2t72oep2o5Jj
</commit_message>
<xml_diff>
--- a/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
+++ b/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L204"/>
+  <dimension ref="A1:L209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -502,7 +502,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 7:45 PM CT · every item numbered · DONE only with live proof</t>
+          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 8:15 PM CT · every item numbered · DONE only with live proof</t>
         </is>
       </c>
     </row>
@@ -12003,6 +12003,282 @@
       </c>
       <c r="K204" s="3" t="inlineStr"/>
       <c r="L204" s="3" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="3" t="n">
+        <v>203</v>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>F · Money tie-outs</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>Linkage</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="inlineStr">
+        <is>
+          <t>Linkage gate red (verify-every-load-born-posting-carries-its-load) blocks every money push</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="inlineStr">
+        <is>
+          <t>uncapped prod: 43 discount legs ($1,976.20) on old load + 12 settlement legs on 4 settlements</t>
+        </is>
+      </c>
+      <c r="F205" s="3" t="inlineStr">
+        <is>
+          <t>AUTH-453 / AUTH-454 repairs built (CC-2 #27384) but never run on prod</t>
+        </is>
+      </c>
+      <c r="G205" s="3" t="inlineStr">
+        <is>
+          <t>fork rehearsal then prod, TB 0 before/after</t>
+        </is>
+      </c>
+      <c r="H205" s="3" t="inlineStr">
+        <is>
+          <t>LEAD</t>
+        </is>
+      </c>
+      <c r="I205" s="3" t="inlineStr">
+        <is>
+          <t>443.287</t>
+        </is>
+      </c>
+      <c r="J205" s="7" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K205" s="3" t="inlineStr">
+        <is>
+          <t>fork br-bitter-lab: AUTH-454 COMMITTED 5 settlements TB 0, postings 7091=7091; AUTH-453 running</t>
+        </is>
+      </c>
+      <c r="L205" s="3" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="n">
+        <v>204</v>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>F · Money tie-outs</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>Fuel</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="inlineStr">
+        <is>
+          <t>Statement card discount / difference is a separate expense with NO link to its receipt; copies the load once, never follows a move</t>
+        </is>
+      </c>
+      <c r="E206" s="3" t="inlineStr">
+        <is>
+          <t>receipt id only in memo (also the no-internal-payload red)</t>
+        </is>
+      </c>
+      <c r="F206" s="3" t="inlineStr">
+        <is>
+          <t>child document not linked to parent; move paths select by fuel link</t>
+        </is>
+      </c>
+      <c r="G206" s="3" t="inlineStr">
+        <is>
+          <t>parent_expense_id + source link; one moveExpenseFamilyToLoad; guard child-follows-parent</t>
+        </is>
+      </c>
+      <c r="H206" s="3" t="inlineStr">
+        <is>
+          <t>CC-2</t>
+        </is>
+      </c>
+      <c r="I206" s="3" t="inlineStr">
+        <is>
+          <t>443.288-A</t>
+        </is>
+      </c>
+      <c r="J206" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K206" s="3" t="inlineStr">
+        <is>
+          <t>owner ruling 443.288 10-23 7:59 PM</t>
+        </is>
+      </c>
+      <c r="L206" s="3" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="3" t="n">
+        <v>205</v>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="inlineStr">
+        <is>
+          <t>OWNER: every expense-to-load assignment confirmed by dispatcher or closer — always</t>
+        </is>
+      </c>
+      <c r="E207" s="3" t="inlineStr">
+        <is>
+          <t>10-23 7:59 PM CT</t>
+        </is>
+      </c>
+      <c r="F207" s="3" t="inlineStr">
+        <is>
+          <t>machine writers set the load as final today</t>
+        </is>
+      </c>
+      <c r="G207" s="3" t="inlineStr">
+        <is>
+          <t>load_confirmation proposed|confirmed; confirm engine; settlement close refuses proposed</t>
+        </is>
+      </c>
+      <c r="H207" s="3" t="inlineStr">
+        <is>
+          <t>CC-2</t>
+        </is>
+      </c>
+      <c r="I207" s="3" t="inlineStr">
+        <is>
+          <t>443.288-B</t>
+        </is>
+      </c>
+      <c r="J207" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K207" s="3" t="inlineStr">
+        <is>
+          <t>docs/bus/lead/OWNER-RULING-443.288-...md</t>
+        </is>
+      </c>
+      <c r="L207" s="3" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="3" t="n">
+        <v>206</v>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>Dispatch / Settlements</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="inlineStr">
+        <is>
+          <t>Expense load confirmations queue (Dispatch + Settlements Close), multi-select, bulk confirm</t>
+        </is>
+      </c>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F208" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G208" s="3" t="inlineStr">
+        <is>
+          <t>V3 board, two-way links</t>
+        </is>
+      </c>
+      <c r="H208" s="3" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="I208" s="3" t="inlineStr">
+        <is>
+          <t>443.288-C</t>
+        </is>
+      </c>
+      <c r="J208" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K208" s="3" t="inlineStr">
+        <is>
+          <t>after 443.288-B route</t>
+        </is>
+      </c>
+      <c r="L208" s="3" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="3" t="n">
+        <v>207</v>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>E · Main static reds</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>Guards</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="inlineStr">
+        <is>
+          <t>Guards for 443.288 (child follows parent, no machine-final load, close refuses proposed, family moves)</t>
+        </is>
+      </c>
+      <c r="E209" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F209" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G209" s="3" t="inlineStr">
+        <is>
+          <t>failing plants; wired with each change</t>
+        </is>
+      </c>
+      <c r="H209" s="3" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="I209" s="3" t="inlineStr">
+        <is>
+          <t>443.288-D</t>
+        </is>
+      </c>
+      <c r="J209" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K209" s="3" t="inlineStr"/>
+      <c r="L209" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:L201"/>

</xml_diff>

<commit_message>
FINDING: N/A LANE: NON-FINANCIAL — LEAD 443.292: register 9:20 PM CT — owner 8:52 PM issues 212-221 measured + 203/201 progress, 208-211
Docs only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0112DqKNUusL2t72oep2o5Jj
</commit_message>
<xml_diff>
--- a/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
+++ b/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L209"/>
+  <dimension ref="A1:L223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -502,7 +502,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 8:15 PM CT · every item numbered · DONE only with live proof</t>
+          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 9:20 PM CT · every item numbered · DONE only with live proof</t>
         </is>
       </c>
     </row>
@@ -11947,7 +11947,7 @@
       </c>
       <c r="K203" s="3" t="inlineStr">
         <is>
-          <t>CC-2: dashboard-connectivity, sweep-pre-list, test-provider; CC-3: partial-optional-chain, unselected-boxes</t>
+          <t>9:00 PM main: 4 of 6 green; left verify-settlement-sweep-pre-list, verify-no-internal-payload-in-notes (CC-2)</t>
         </is>
       </c>
       <c r="L203" s="3" t="n"/>
@@ -12055,7 +12055,7 @@
       </c>
       <c r="K205" s="3" t="inlineStr">
         <is>
-          <t>fork br-bitter-lab: AUTH-454 COMMITTED 5 settlements TB 0, postings 7091=7091; AUTH-453 running</t>
+          <t>AUTH-454 COMMITTED on prod (5 headers, TB 0, 7091=7091); AUTH-453 running on prod (owner OK 8:42 PM); fork: uncapped guard exit 0</t>
         </is>
       </c>
       <c r="L205" s="3" t="n"/>
@@ -12279,6 +12279,750 @@
       </c>
       <c r="K209" s="3" t="inlineStr"/>
       <c r="L209" s="3" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="n">
+        <v>208</v>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>E · Main static reds</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="inlineStr">
+        <is>
+          <t>Main CI red at verify:arch-design (/insurance, Fuel Planner settings + Expense mapping)</t>
+        </is>
+      </c>
+      <c r="E210" s="3" t="inlineStr">
+        <is>
+          <t>nothing removed: /insurance/* route; V3Panel titles</t>
+        </is>
+      </c>
+      <c r="F210" s="3" t="inlineStr">
+        <is>
+          <t>reader read literals + h3 only</t>
+        </is>
+      </c>
+      <c r="G210" s="3" t="inlineStr">
+        <is>
+          <t>reader credits splat bases + V3 panel titles, plants</t>
+        </is>
+      </c>
+      <c r="H210" s="3" t="inlineStr">
+        <is>
+          <t>LEAD</t>
+        </is>
+      </c>
+      <c r="I210" s="3" t="inlineStr">
+        <is>
+          <t>443.289</t>
+        </is>
+      </c>
+      <c r="J210" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="K210" s="3" t="inlineStr">
+        <is>
+          <t>#27422 b1192f1e; plants red; CI re-run pending</t>
+        </is>
+      </c>
+      <c r="L210" s="3" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="n">
+        <v>209</v>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>E · Main static reds</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>Guards</t>
+        </is>
+      </c>
+      <c r="D211" s="3" t="inlineStr">
+        <is>
+          <t>107 main static reds outside baseline split by seat</t>
+        </is>
+      </c>
+      <c r="E211" s="3" t="inlineStr">
+        <is>
+          <t>full verify:static 8:35 PM</t>
+        </is>
+      </c>
+      <c r="F211" s="3" t="inlineStr">
+        <is>
+          <t>board merges + stale text guards</t>
+        </is>
+      </c>
+      <c r="G211" s="3" t="inlineStr">
+        <is>
+          <t>fix code or retarget with plants</t>
+        </is>
+      </c>
+      <c r="H211" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="I211" s="3" t="inlineStr">
+        <is>
+          <t>443.290</t>
+        </is>
+      </c>
+      <c r="J211" s="7" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K211" s="3" t="inlineStr">
+        <is>
+          <t>#27407 list; CC-1 #27413/#27416/#27417; Lead 4 Cash Flow in 443.283c</t>
+        </is>
+      </c>
+      <c r="L211" s="3" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="n">
+        <v>210</v>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>E · Guards</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D212" s="3" t="inlineStr">
+        <is>
+          <t>6,266 guard scripts (488 live, ~5,700 source-text, 316 slate-color copies)</t>
+        </is>
+      </c>
+      <c r="E212" s="3" t="inlineStr">
+        <is>
+          <t>census 8:50 PM</t>
+        </is>
+      </c>
+      <c r="F212" s="3" t="inlineStr">
+        <is>
+          <t>one guard per bug, never merged</t>
+        </is>
+      </c>
+      <c r="G212" s="3" t="inlineStr">
+        <is>
+          <t>consolidate: one check per family; text never guards money</t>
+        </is>
+      </c>
+      <c r="H212" s="3" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="I212" s="3" t="inlineStr">
+        <is>
+          <t>443.291</t>
+        </is>
+      </c>
+      <c r="J212" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K212" s="3" t="inlineStr">
+        <is>
+          <t>after Codex filters PR</t>
+        </is>
+      </c>
+      <c r="L212" s="3" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="3" t="n">
+        <v>211</v>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>F · Money tie-outs</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>Cash Flow</t>
+        </is>
+      </c>
+      <c r="D213" s="3" t="inlineStr">
+        <is>
+          <t>Actual vs Projected + Manual reverted to pre-board code by #27390</t>
+        </is>
+      </c>
+      <c r="E213" s="3" t="inlineStr">
+        <is>
+          <t>AvP 626→380 lines; 4 KPIs + chart gone</t>
+        </is>
+      </c>
+      <c r="F213" s="3" t="inlineStr">
+        <is>
+          <t>#27390 replaced files with old versions</t>
+        </is>
+      </c>
+      <c r="G213" s="3" t="inlineStr">
+        <is>
+          <t>restore approved boards</t>
+        </is>
+      </c>
+      <c r="H213" s="3" t="inlineStr">
+        <is>
+          <t>LEAD</t>
+        </is>
+      </c>
+      <c r="I213" s="3" t="inlineStr">
+        <is>
+          <t>443.283c</t>
+        </is>
+      </c>
+      <c r="J213" s="7" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K213" s="3" t="inlineStr">
+        <is>
+          <t>162429bd guards + 7/7 tests; push after linkage green</t>
+        </is>
+      </c>
+      <c r="L213" s="3" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="3" t="n">
+        <v>212</v>
+      </c>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D214" s="3" t="inlineStr">
+        <is>
+          <t>Settlement number: P-number shown; real series not assigned by our system</t>
+        </is>
+      </c>
+      <c r="E214" s="3" t="inlineStr">
+        <is>
+          <t>82 numbered (max 5851), 12 not; 5 closed today without number</t>
+        </is>
+      </c>
+      <c r="F214" s="3" t="inlineStr">
+        <is>
+          <t>close engine never assigns</t>
+        </is>
+      </c>
+      <c r="G214" s="3" t="inlineStr">
+        <is>
+          <t>auto-assign at close, next in series, shown everywhere</t>
+        </is>
+      </c>
+      <c r="H214" s="3" t="inlineStr">
+        <is>
+          <t>CC-1</t>
+        </is>
+      </c>
+      <c r="I214" s="3" t="inlineStr">
+        <is>
+          <t>443.292-A</t>
+        </is>
+      </c>
+      <c r="J214" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K214" s="3" t="inlineStr"/>
+      <c r="L214" s="3" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="3" t="n">
+        <v>213</v>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D215" s="3" t="inlineStr">
+        <is>
+          <t>Tour dates wrong (P-0114 10/20→10/20; real 10/16→10/23)</t>
+        </is>
+      </c>
+      <c r="E215" s="3" t="inlineStr">
+        <is>
+          <t>open headers period = creation day; UTC midnight renders a day early</t>
+        </is>
+      </c>
+      <c r="F215" s="3" t="inlineStr">
+        <is>
+          <t>writer stamps creation date</t>
+        </is>
+      </c>
+      <c r="G215" s="3" t="inlineStr">
+        <is>
+          <t>first pickup → last delivery, DATE type, re-derive 12</t>
+        </is>
+      </c>
+      <c r="H215" s="3" t="inlineStr">
+        <is>
+          <t>CC-1</t>
+        </is>
+      </c>
+      <c r="I215" s="3" t="inlineStr">
+        <is>
+          <t>443.292-B</t>
+        </is>
+      </c>
+      <c r="J215" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K215" s="3" t="inlineStr"/>
+      <c r="L215" s="3" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="3" t="n">
+        <v>214</v>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D216" s="3" t="inlineStr">
+        <is>
+          <t>Settlements tab week list: closed show Open; duplicate empty driver rows</t>
+        </is>
+      </c>
+      <c r="E216" s="3" t="inlineStr">
+        <is>
+          <t>P-0107 closed reads Open</t>
+        </is>
+      </c>
+      <c r="F216" s="3" t="inlineStr">
+        <is>
+          <t>wrong status field</t>
+        </is>
+      </c>
+      <c r="G216" s="3" t="inlineStr">
+        <is>
+          <t>status + payment status columns</t>
+        </is>
+      </c>
+      <c r="H216" s="3" t="inlineStr">
+        <is>
+          <t>CC-1</t>
+        </is>
+      </c>
+      <c r="I216" s="3" t="inlineStr">
+        <is>
+          <t>443.292-C</t>
+        </is>
+      </c>
+      <c r="J216" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K216" s="3" t="inlineStr"/>
+      <c r="L216" s="3" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="3" t="n">
+        <v>215</v>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D217" s="3" t="inlineStr">
+        <is>
+          <t>Escrow register: all same date/source, no load numbers; escrow is per load</t>
+        </is>
+      </c>
+      <c r="E217" s="3" t="inlineStr">
+        <is>
+          <t>escrow_ledger 58 rows: load 0, settlement 2</t>
+        </is>
+      </c>
+      <c r="F217" s="3" t="inlineStr">
+        <is>
+          <t>close engine writes no load/settlement</t>
+        </is>
+      </c>
+      <c r="G217" s="3" t="inlineStr">
+        <is>
+          <t>per-load rows + backfill; Date·Settlement#·Load#</t>
+        </is>
+      </c>
+      <c r="H217" s="3" t="inlineStr">
+        <is>
+          <t>CC-1</t>
+        </is>
+      </c>
+      <c r="I217" s="3" t="inlineStr">
+        <is>
+          <t>443.292-D</t>
+        </is>
+      </c>
+      <c r="J217" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K217" s="3" t="inlineStr"/>
+      <c r="L217" s="3" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="B218" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D218" s="3" t="inlineStr">
+        <is>
+          <t>Bill Payments shows driver escrows — not bill payments</t>
+        </is>
+      </c>
+      <c r="E218" s="3" t="inlineStr">
+        <is>
+          <t>218 rows $7,303.21 all settlement deductions; 0 cash</t>
+        </is>
+      </c>
+      <c r="F218" s="3" t="inlineStr">
+        <is>
+          <t>deduction recorded as bill_payment</t>
+        </is>
+      </c>
+      <c r="G218" s="3" t="inlineStr">
+        <is>
+          <t>deduction application kind; Bill Payments = cash only; A/P still 126,443.92</t>
+        </is>
+      </c>
+      <c r="H218" s="3" t="inlineStr">
+        <is>
+          <t>CC-1</t>
+        </is>
+      </c>
+      <c r="I218" s="3" t="inlineStr">
+        <is>
+          <t>443.292-E</t>
+        </is>
+      </c>
+      <c r="J218" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K218" s="3" t="inlineStr"/>
+      <c r="L218" s="3" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="3" t="n">
+        <v>217</v>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D219" s="3" t="inlineStr">
+        <is>
+          <t>Empty closed settlements P-0123, P-0124 ($0, 0 lines)</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="inlineStr">
+        <is>
+          <t>closed 10/23</t>
+        </is>
+      </c>
+      <c r="F219" s="3" t="inlineStr">
+        <is>
+          <t>close engine allows empty</t>
+        </is>
+      </c>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>refuse empty; void both via engine</t>
+        </is>
+      </c>
+      <c r="H219" s="3" t="inlineStr">
+        <is>
+          <t>CC-1</t>
+        </is>
+      </c>
+      <c r="I219" s="3" t="inlineStr">
+        <is>
+          <t>443.292-F</t>
+        </is>
+      </c>
+      <c r="J219" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K219" s="3" t="inlineStr"/>
+      <c r="L219" s="3" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="3" t="n">
+        <v>218</v>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D220" s="3" t="inlineStr">
+        <is>
+          <t>Statement must match the owner settlement document (5753 format): loads+stops+dates, fuel, expenses, per-load deductions, P&amp;L</t>
+        </is>
+      </c>
+      <c r="E220" s="3" t="inlineStr">
+        <is>
+          <t>P-0114 statement shows no dates, $0 deductions line, fuel —</t>
+        </is>
+      </c>
+      <c r="F220" s="3" t="inlineStr">
+        <is>
+          <t>summary page, not the document</t>
+        </is>
+      </c>
+      <c r="G220" s="3" t="inlineStr">
+        <is>
+          <t>8 sections as Company/Driver_Settlement_5753</t>
+        </is>
+      </c>
+      <c r="H220" s="3" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="I220" s="3" t="inlineStr">
+        <is>
+          <t>443.293-A</t>
+        </is>
+      </c>
+      <c r="J220" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K220" s="3" t="inlineStr"/>
+      <c r="L220" s="3" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="3" t="n">
+        <v>219</v>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>Dispatch / Settlements</t>
+        </is>
+      </c>
+      <c r="D221" s="3" t="inlineStr">
+        <is>
+          <t>Settlement Close: what it does; should be a button in Dispatch</t>
+        </is>
+      </c>
+      <c r="E221" s="3" t="inlineStr">
+        <is>
+          <t>it is the 7-step close wizard</t>
+        </is>
+      </c>
+      <c r="F221" s="3" t="inlineStr">
+        <is>
+          <t>only reachable in Settlements</t>
+        </is>
+      </c>
+      <c r="G221" s="3" t="inlineStr">
+        <is>
+          <t>Close settlement button in Dispatch opens the same wizard; tab = closer queue</t>
+        </is>
+      </c>
+      <c r="H221" s="3" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="I221" s="3" t="inlineStr">
+        <is>
+          <t>443.293-B</t>
+        </is>
+      </c>
+      <c r="J221" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K221" s="3" t="inlineStr"/>
+      <c r="L221" s="3" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D222" s="3" t="inlineStr">
+        <is>
+          <t>Inspect every Accounting tab; only Bills first tab is right</t>
+        </is>
+      </c>
+      <c r="E222" s="3" t="inlineStr">
+        <is>
+          <t>owner 8:52 PM</t>
+        </is>
+      </c>
+      <c r="F222" s="3" t="inlineStr">
+        <is>
+          <t>tabs not on V3 board grammar</t>
+        </is>
+      </c>
+      <c r="G222" s="3" t="inlineStr">
+        <is>
+          <t>every tab to Bills-first-tab grammar, screenshots</t>
+        </is>
+      </c>
+      <c r="H222" s="3" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="I222" s="3" t="inlineStr">
+        <is>
+          <t>443.293-C</t>
+        </is>
+      </c>
+      <c r="J222" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K222" s="3" t="inlineStr"/>
+      <c r="L222" s="3" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="3" t="n">
+        <v>221</v>
+      </c>
+      <c r="B223" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>All modules</t>
+        </is>
+      </c>
+      <c r="D223" s="3" t="inlineStr">
+        <is>
+          <t>Override: one reasons catalog + one button app-wide; owner/accountant confirm only; others dropdown; no typing</t>
+        </is>
+      </c>
+      <c r="E223" s="3" t="inlineStr">
+        <is>
+          <t>67 files with ad-hoc override reasons</t>
+        </is>
+      </c>
+      <c r="F223" s="3" t="inlineStr">
+        <is>
+          <t>no shared catalog/engine</t>
+        </is>
+      </c>
+      <c r="G223" s="3" t="inlineStr">
+        <is>
+          <t>catalogs.override_reasons + recordOverride + OverrideButton; replace 67</t>
+        </is>
+      </c>
+      <c r="H223" s="3" t="inlineStr">
+        <is>
+          <t>CC-3</t>
+        </is>
+      </c>
+      <c r="I223" s="3" t="inlineStr">
+        <is>
+          <t>443.294</t>
+        </is>
+      </c>
+      <c r="J223" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K223" s="3" t="inlineStr"/>
+      <c r="L223" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:L201"/>

</xml_diff>

<commit_message>
FINDING: N/A LANE: NON-FINANCIAL — LEAD 443.292: register 9:20 PM CT — owner 8:52 PM issues 212-221 measured + 203/201 progress, 208-211 (#27426)
Docs only.


Claude-Session: https://claude.ai/code/session_0112DqKNUusL2t72oep2o5Jj

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
+++ b/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L209"/>
+  <dimension ref="A1:L223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -502,7 +502,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 8:15 PM CT · every item numbered · DONE only with live proof</t>
+          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 9:20 PM CT · every item numbered · DONE only with live proof</t>
         </is>
       </c>
     </row>
@@ -11947,7 +11947,7 @@
       </c>
       <c r="K203" s="3" t="inlineStr">
         <is>
-          <t>CC-2: dashboard-connectivity, sweep-pre-list, test-provider; CC-3: partial-optional-chain, unselected-boxes</t>
+          <t>9:00 PM main: 4 of 6 green; left verify-settlement-sweep-pre-list, verify-no-internal-payload-in-notes (CC-2)</t>
         </is>
       </c>
       <c r="L203" s="3" t="n"/>
@@ -12055,7 +12055,7 @@
       </c>
       <c r="K205" s="3" t="inlineStr">
         <is>
-          <t>fork br-bitter-lab: AUTH-454 COMMITTED 5 settlements TB 0, postings 7091=7091; AUTH-453 running</t>
+          <t>AUTH-454 COMMITTED on prod (5 headers, TB 0, 7091=7091); AUTH-453 running on prod (owner OK 8:42 PM); fork: uncapped guard exit 0</t>
         </is>
       </c>
       <c r="L205" s="3" t="n"/>
@@ -12279,6 +12279,750 @@
       </c>
       <c r="K209" s="3" t="inlineStr"/>
       <c r="L209" s="3" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="n">
+        <v>208</v>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>E · Main static reds</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="inlineStr">
+        <is>
+          <t>Main CI red at verify:arch-design (/insurance, Fuel Planner settings + Expense mapping)</t>
+        </is>
+      </c>
+      <c r="E210" s="3" t="inlineStr">
+        <is>
+          <t>nothing removed: /insurance/* route; V3Panel titles</t>
+        </is>
+      </c>
+      <c r="F210" s="3" t="inlineStr">
+        <is>
+          <t>reader read literals + h3 only</t>
+        </is>
+      </c>
+      <c r="G210" s="3" t="inlineStr">
+        <is>
+          <t>reader credits splat bases + V3 panel titles, plants</t>
+        </is>
+      </c>
+      <c r="H210" s="3" t="inlineStr">
+        <is>
+          <t>LEAD</t>
+        </is>
+      </c>
+      <c r="I210" s="3" t="inlineStr">
+        <is>
+          <t>443.289</t>
+        </is>
+      </c>
+      <c r="J210" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="K210" s="3" t="inlineStr">
+        <is>
+          <t>#27422 b1192f1e; plants red; CI re-run pending</t>
+        </is>
+      </c>
+      <c r="L210" s="3" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="n">
+        <v>209</v>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>E · Main static reds</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>Guards</t>
+        </is>
+      </c>
+      <c r="D211" s="3" t="inlineStr">
+        <is>
+          <t>107 main static reds outside baseline split by seat</t>
+        </is>
+      </c>
+      <c r="E211" s="3" t="inlineStr">
+        <is>
+          <t>full verify:static 8:35 PM</t>
+        </is>
+      </c>
+      <c r="F211" s="3" t="inlineStr">
+        <is>
+          <t>board merges + stale text guards</t>
+        </is>
+      </c>
+      <c r="G211" s="3" t="inlineStr">
+        <is>
+          <t>fix code or retarget with plants</t>
+        </is>
+      </c>
+      <c r="H211" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="I211" s="3" t="inlineStr">
+        <is>
+          <t>443.290</t>
+        </is>
+      </c>
+      <c r="J211" s="7" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K211" s="3" t="inlineStr">
+        <is>
+          <t>#27407 list; CC-1 #27413/#27416/#27417; Lead 4 Cash Flow in 443.283c</t>
+        </is>
+      </c>
+      <c r="L211" s="3" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="n">
+        <v>210</v>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>E · Guards</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D212" s="3" t="inlineStr">
+        <is>
+          <t>6,266 guard scripts (488 live, ~5,700 source-text, 316 slate-color copies)</t>
+        </is>
+      </c>
+      <c r="E212" s="3" t="inlineStr">
+        <is>
+          <t>census 8:50 PM</t>
+        </is>
+      </c>
+      <c r="F212" s="3" t="inlineStr">
+        <is>
+          <t>one guard per bug, never merged</t>
+        </is>
+      </c>
+      <c r="G212" s="3" t="inlineStr">
+        <is>
+          <t>consolidate: one check per family; text never guards money</t>
+        </is>
+      </c>
+      <c r="H212" s="3" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="I212" s="3" t="inlineStr">
+        <is>
+          <t>443.291</t>
+        </is>
+      </c>
+      <c r="J212" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K212" s="3" t="inlineStr">
+        <is>
+          <t>after Codex filters PR</t>
+        </is>
+      </c>
+      <c r="L212" s="3" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="3" t="n">
+        <v>211</v>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>F · Money tie-outs</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>Cash Flow</t>
+        </is>
+      </c>
+      <c r="D213" s="3" t="inlineStr">
+        <is>
+          <t>Actual vs Projected + Manual reverted to pre-board code by #27390</t>
+        </is>
+      </c>
+      <c r="E213" s="3" t="inlineStr">
+        <is>
+          <t>AvP 626→380 lines; 4 KPIs + chart gone</t>
+        </is>
+      </c>
+      <c r="F213" s="3" t="inlineStr">
+        <is>
+          <t>#27390 replaced files with old versions</t>
+        </is>
+      </c>
+      <c r="G213" s="3" t="inlineStr">
+        <is>
+          <t>restore approved boards</t>
+        </is>
+      </c>
+      <c r="H213" s="3" t="inlineStr">
+        <is>
+          <t>LEAD</t>
+        </is>
+      </c>
+      <c r="I213" s="3" t="inlineStr">
+        <is>
+          <t>443.283c</t>
+        </is>
+      </c>
+      <c r="J213" s="7" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K213" s="3" t="inlineStr">
+        <is>
+          <t>162429bd guards + 7/7 tests; push after linkage green</t>
+        </is>
+      </c>
+      <c r="L213" s="3" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="3" t="n">
+        <v>212</v>
+      </c>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D214" s="3" t="inlineStr">
+        <is>
+          <t>Settlement number: P-number shown; real series not assigned by our system</t>
+        </is>
+      </c>
+      <c r="E214" s="3" t="inlineStr">
+        <is>
+          <t>82 numbered (max 5851), 12 not; 5 closed today without number</t>
+        </is>
+      </c>
+      <c r="F214" s="3" t="inlineStr">
+        <is>
+          <t>close engine never assigns</t>
+        </is>
+      </c>
+      <c r="G214" s="3" t="inlineStr">
+        <is>
+          <t>auto-assign at close, next in series, shown everywhere</t>
+        </is>
+      </c>
+      <c r="H214" s="3" t="inlineStr">
+        <is>
+          <t>CC-1</t>
+        </is>
+      </c>
+      <c r="I214" s="3" t="inlineStr">
+        <is>
+          <t>443.292-A</t>
+        </is>
+      </c>
+      <c r="J214" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K214" s="3" t="inlineStr"/>
+      <c r="L214" s="3" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="3" t="n">
+        <v>213</v>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D215" s="3" t="inlineStr">
+        <is>
+          <t>Tour dates wrong (P-0114 10/20→10/20; real 10/16→10/23)</t>
+        </is>
+      </c>
+      <c r="E215" s="3" t="inlineStr">
+        <is>
+          <t>open headers period = creation day; UTC midnight renders a day early</t>
+        </is>
+      </c>
+      <c r="F215" s="3" t="inlineStr">
+        <is>
+          <t>writer stamps creation date</t>
+        </is>
+      </c>
+      <c r="G215" s="3" t="inlineStr">
+        <is>
+          <t>first pickup → last delivery, DATE type, re-derive 12</t>
+        </is>
+      </c>
+      <c r="H215" s="3" t="inlineStr">
+        <is>
+          <t>CC-1</t>
+        </is>
+      </c>
+      <c r="I215" s="3" t="inlineStr">
+        <is>
+          <t>443.292-B</t>
+        </is>
+      </c>
+      <c r="J215" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K215" s="3" t="inlineStr"/>
+      <c r="L215" s="3" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="3" t="n">
+        <v>214</v>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D216" s="3" t="inlineStr">
+        <is>
+          <t>Settlements tab week list: closed show Open; duplicate empty driver rows</t>
+        </is>
+      </c>
+      <c r="E216" s="3" t="inlineStr">
+        <is>
+          <t>P-0107 closed reads Open</t>
+        </is>
+      </c>
+      <c r="F216" s="3" t="inlineStr">
+        <is>
+          <t>wrong status field</t>
+        </is>
+      </c>
+      <c r="G216" s="3" t="inlineStr">
+        <is>
+          <t>status + payment status columns</t>
+        </is>
+      </c>
+      <c r="H216" s="3" t="inlineStr">
+        <is>
+          <t>CC-1</t>
+        </is>
+      </c>
+      <c r="I216" s="3" t="inlineStr">
+        <is>
+          <t>443.292-C</t>
+        </is>
+      </c>
+      <c r="J216" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K216" s="3" t="inlineStr"/>
+      <c r="L216" s="3" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="3" t="n">
+        <v>215</v>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D217" s="3" t="inlineStr">
+        <is>
+          <t>Escrow register: all same date/source, no load numbers; escrow is per load</t>
+        </is>
+      </c>
+      <c r="E217" s="3" t="inlineStr">
+        <is>
+          <t>escrow_ledger 58 rows: load 0, settlement 2</t>
+        </is>
+      </c>
+      <c r="F217" s="3" t="inlineStr">
+        <is>
+          <t>close engine writes no load/settlement</t>
+        </is>
+      </c>
+      <c r="G217" s="3" t="inlineStr">
+        <is>
+          <t>per-load rows + backfill; Date·Settlement#·Load#</t>
+        </is>
+      </c>
+      <c r="H217" s="3" t="inlineStr">
+        <is>
+          <t>CC-1</t>
+        </is>
+      </c>
+      <c r="I217" s="3" t="inlineStr">
+        <is>
+          <t>443.292-D</t>
+        </is>
+      </c>
+      <c r="J217" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K217" s="3" t="inlineStr"/>
+      <c r="L217" s="3" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="B218" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D218" s="3" t="inlineStr">
+        <is>
+          <t>Bill Payments shows driver escrows — not bill payments</t>
+        </is>
+      </c>
+      <c r="E218" s="3" t="inlineStr">
+        <is>
+          <t>218 rows $7,303.21 all settlement deductions; 0 cash</t>
+        </is>
+      </c>
+      <c r="F218" s="3" t="inlineStr">
+        <is>
+          <t>deduction recorded as bill_payment</t>
+        </is>
+      </c>
+      <c r="G218" s="3" t="inlineStr">
+        <is>
+          <t>deduction application kind; Bill Payments = cash only; A/P still 126,443.92</t>
+        </is>
+      </c>
+      <c r="H218" s="3" t="inlineStr">
+        <is>
+          <t>CC-1</t>
+        </is>
+      </c>
+      <c r="I218" s="3" t="inlineStr">
+        <is>
+          <t>443.292-E</t>
+        </is>
+      </c>
+      <c r="J218" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K218" s="3" t="inlineStr"/>
+      <c r="L218" s="3" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="3" t="n">
+        <v>217</v>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D219" s="3" t="inlineStr">
+        <is>
+          <t>Empty closed settlements P-0123, P-0124 ($0, 0 lines)</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="inlineStr">
+        <is>
+          <t>closed 10/23</t>
+        </is>
+      </c>
+      <c r="F219" s="3" t="inlineStr">
+        <is>
+          <t>close engine allows empty</t>
+        </is>
+      </c>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>refuse empty; void both via engine</t>
+        </is>
+      </c>
+      <c r="H219" s="3" t="inlineStr">
+        <is>
+          <t>CC-1</t>
+        </is>
+      </c>
+      <c r="I219" s="3" t="inlineStr">
+        <is>
+          <t>443.292-F</t>
+        </is>
+      </c>
+      <c r="J219" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K219" s="3" t="inlineStr"/>
+      <c r="L219" s="3" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="3" t="n">
+        <v>218</v>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D220" s="3" t="inlineStr">
+        <is>
+          <t>Statement must match the owner settlement document (5753 format): loads+stops+dates, fuel, expenses, per-load deductions, P&amp;L</t>
+        </is>
+      </c>
+      <c r="E220" s="3" t="inlineStr">
+        <is>
+          <t>P-0114 statement shows no dates, $0 deductions line, fuel —</t>
+        </is>
+      </c>
+      <c r="F220" s="3" t="inlineStr">
+        <is>
+          <t>summary page, not the document</t>
+        </is>
+      </c>
+      <c r="G220" s="3" t="inlineStr">
+        <is>
+          <t>8 sections as Company/Driver_Settlement_5753</t>
+        </is>
+      </c>
+      <c r="H220" s="3" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="I220" s="3" t="inlineStr">
+        <is>
+          <t>443.293-A</t>
+        </is>
+      </c>
+      <c r="J220" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K220" s="3" t="inlineStr"/>
+      <c r="L220" s="3" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="3" t="n">
+        <v>219</v>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>Dispatch / Settlements</t>
+        </is>
+      </c>
+      <c r="D221" s="3" t="inlineStr">
+        <is>
+          <t>Settlement Close: what it does; should be a button in Dispatch</t>
+        </is>
+      </c>
+      <c r="E221" s="3" t="inlineStr">
+        <is>
+          <t>it is the 7-step close wizard</t>
+        </is>
+      </c>
+      <c r="F221" s="3" t="inlineStr">
+        <is>
+          <t>only reachable in Settlements</t>
+        </is>
+      </c>
+      <c r="G221" s="3" t="inlineStr">
+        <is>
+          <t>Close settlement button in Dispatch opens the same wizard; tab = closer queue</t>
+        </is>
+      </c>
+      <c r="H221" s="3" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="I221" s="3" t="inlineStr">
+        <is>
+          <t>443.293-B</t>
+        </is>
+      </c>
+      <c r="J221" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K221" s="3" t="inlineStr"/>
+      <c r="L221" s="3" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D222" s="3" t="inlineStr">
+        <is>
+          <t>Inspect every Accounting tab; only Bills first tab is right</t>
+        </is>
+      </c>
+      <c r="E222" s="3" t="inlineStr">
+        <is>
+          <t>owner 8:52 PM</t>
+        </is>
+      </c>
+      <c r="F222" s="3" t="inlineStr">
+        <is>
+          <t>tabs not on V3 board grammar</t>
+        </is>
+      </c>
+      <c r="G222" s="3" t="inlineStr">
+        <is>
+          <t>every tab to Bills-first-tab grammar, screenshots</t>
+        </is>
+      </c>
+      <c r="H222" s="3" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="I222" s="3" t="inlineStr">
+        <is>
+          <t>443.293-C</t>
+        </is>
+      </c>
+      <c r="J222" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K222" s="3" t="inlineStr"/>
+      <c r="L222" s="3" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="3" t="n">
+        <v>221</v>
+      </c>
+      <c r="B223" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>All modules</t>
+        </is>
+      </c>
+      <c r="D223" s="3" t="inlineStr">
+        <is>
+          <t>Override: one reasons catalog + one button app-wide; owner/accountant confirm only; others dropdown; no typing</t>
+        </is>
+      </c>
+      <c r="E223" s="3" t="inlineStr">
+        <is>
+          <t>67 files with ad-hoc override reasons</t>
+        </is>
+      </c>
+      <c r="F223" s="3" t="inlineStr">
+        <is>
+          <t>no shared catalog/engine</t>
+        </is>
+      </c>
+      <c r="G223" s="3" t="inlineStr">
+        <is>
+          <t>catalogs.override_reasons + recordOverride + OverrideButton; replace 67</t>
+        </is>
+      </c>
+      <c r="H223" s="3" t="inlineStr">
+        <is>
+          <t>CC-3</t>
+        </is>
+      </c>
+      <c r="I223" s="3" t="inlineStr">
+        <is>
+          <t>443.294</t>
+        </is>
+      </c>
+      <c r="J223" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K223" s="3" t="inlineStr"/>
+      <c r="L223" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:L201"/>

</xml_diff>

<commit_message>
FINDING: N/A LANE: NON-FINANCIAL — LEAD 443.297: code-complete mode — register seats reassigned (CC-1 38, CC-2 25, CC-3 22, Cursor 77, Codex 27), rows 222-224, and all 10-23 coder boxes
Docs only: docs/bus/lead/LEAD-PENDING-REGISTER.xlsx/.md + docs/bus/lead/boxes/2026-10-23/ (40 coder instruction boxes).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0112DqKNUusL2t72oep2o5Jj
</commit_message>
<xml_diff>
--- a/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
+++ b/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L223"/>
+  <dimension ref="A1:L226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -502,7 +502,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 9:20 PM CT · every item numbered · DONE only with live proof</t>
+          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 10:15 PM CT · CODE-COMPLETE MODE (owner 9:40 PM) · deadline 10-24 10:00 AM CT</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>LEAD/CC-3</t>
+          <t>LEAD</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>CC-2 + CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>CURSOR/CC-1</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>CC-3/CURSOR</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>CURSOR/CODEX/CC-3</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>CURSOR + CC-1</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>CODEX (guard) + CURSOR (pages)</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -2948,7 +2948,7 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
@@ -3288,7 +3288,7 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
@@ -3516,7 +3516,7 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -4116,7 +4116,7 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -4376,7 +4376,7 @@
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>CC-2 + OWNER</t>
+          <t>CC-2</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>CC-2 + OWNER</t>
+          <t>CC-2</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>CC-2 + OWNER</t>
+          <t>CC-2</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>CC-2</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I100" s="3" t="inlineStr">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>CC-2</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I102" s="3" t="inlineStr">
@@ -6132,7 +6132,7 @@
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I104" s="3" t="inlineStr">
@@ -6188,7 +6188,7 @@
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I105" s="3" t="inlineStr">
@@ -6472,7 +6472,7 @@
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
-          <t>CC-3</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I110" s="3" t="inlineStr">
@@ -6584,7 +6584,7 @@
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>CODEX/CC-3</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I112" s="3" t="inlineStr">
@@ -6640,7 +6640,7 @@
       </c>
       <c r="H113" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I113" s="3" t="inlineStr">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
-          <t>CC-2</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I114" s="3" t="inlineStr">
@@ -6800,7 +6800,7 @@
       <c r="G116" s="3" t="inlineStr"/>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I116" s="3" t="inlineStr">
@@ -6844,7 +6844,7 @@
       <c r="G117" s="3" t="inlineStr"/>
       <c r="H117" s="3" t="inlineStr">
         <is>
-          <t>CC-2/CC-3</t>
+          <t>CC-2</t>
         </is>
       </c>
       <c r="I117" s="3" t="inlineStr">
@@ -6984,7 +6984,7 @@
       <c r="G120" s="3" t="inlineStr"/>
       <c r="H120" s="3" t="inlineStr">
         <is>
-          <t>CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I120" s="3" t="inlineStr">
@@ -7028,7 +7028,7 @@
       <c r="G121" s="3" t="inlineStr"/>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I121" s="3" t="inlineStr">
@@ -7204,7 +7204,7 @@
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -7384,7 +7384,7 @@
       </c>
       <c r="H127" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I127" s="3" t="inlineStr">
@@ -8344,7 +8344,7 @@
       </c>
       <c r="H143" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I143" s="3" t="inlineStr">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H147" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I147" s="3" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="H148" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I148" s="3" t="inlineStr">
@@ -8884,7 +8884,7 @@
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I152" s="3" t="inlineStr">
@@ -9004,7 +9004,7 @@
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="H155" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I155" s="3" t="inlineStr">
@@ -9124,7 +9124,7 @@
       </c>
       <c r="H156" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I156" s="3" t="inlineStr">
@@ -9184,7 +9184,7 @@
       </c>
       <c r="H157" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I157" s="3" t="inlineStr">
@@ -9244,7 +9244,7 @@
       </c>
       <c r="H158" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I158" s="3" t="inlineStr">
@@ -9304,7 +9304,7 @@
       </c>
       <c r="H159" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I159" s="3" t="inlineStr">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="H160" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I160" s="3" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="H161" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I161" s="3" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="H165" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I165" s="3" t="inlineStr">
@@ -9784,7 +9784,7 @@
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -9844,7 +9844,7 @@
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
@@ -9904,7 +9904,7 @@
       </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I169" s="3" t="inlineStr">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I170" s="3" t="inlineStr">
@@ -10204,7 +10204,7 @@
       </c>
       <c r="H174" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I174" s="3" t="inlineStr">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I175" s="3" t="inlineStr">
@@ -10324,7 +10324,7 @@
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I176" s="3" t="inlineStr">
@@ -10444,7 +10444,7 @@
       </c>
       <c r="H178" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I178" s="3" t="inlineStr">
@@ -10804,7 +10804,7 @@
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I184" s="3" t="inlineStr">
@@ -11464,7 +11464,7 @@
       </c>
       <c r="H195" s="3" t="inlineStr">
         <is>
-          <t>Lead assigns</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I195" s="3" t="inlineStr">
@@ -11704,7 +11704,7 @@
       </c>
       <c r="H199" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I199" s="3" t="inlineStr">
@@ -11764,7 +11764,7 @@
       </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I200" s="3" t="inlineStr">
@@ -11820,7 +11820,7 @@
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
-          <t>CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I201" s="3" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>CC-2/CC-3</t>
+          <t>CC-2</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -12055,7 +12055,7 @@
       </c>
       <c r="K205" s="3" t="inlineStr">
         <is>
-          <t>AUTH-454 COMMITTED on prod (5 headers, TB 0, 7091=7091); AUTH-453 running on prod (owner OK 8:42 PM); fork: uncapped guard exit 0</t>
+          <t>AUTH-454 COMMITTED prod (TB 0); AUTH-453 150/241 on prod 10:15 PM, TB 0, retry loop (lock contention)</t>
         </is>
       </c>
       <c r="L205" s="3" t="n"/>
@@ -12372,7 +12372,7 @@
       </c>
       <c r="H211" s="3" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I211" s="3" t="inlineStr">
@@ -13023,6 +13023,170 @@
       </c>
       <c r="K223" s="3" t="inlineStr"/>
       <c r="L223" s="3" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="3" t="n">
+        <v>222</v>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="inlineStr">
+        <is>
+          <t>All modules</t>
+        </is>
+      </c>
+      <c r="D224" s="3" t="inlineStr">
+        <is>
+          <t>Popup standard app-wide + Fuel assignment popup redesign</t>
+        </is>
+      </c>
+      <c r="E224" s="3" t="inlineStr">
+        <is>
+          <t>Modal falls back to 85% width; 140 of 155 popup files pass no size</t>
+        </is>
+      </c>
+      <c r="F224" s="3" t="inlineStr">
+        <is>
+          <t>no width caps except xl</t>
+        </is>
+      </c>
+      <c r="G224" s="3" t="inlineStr">
+        <is>
+          <t>sm 480/md 720/lg 960/xl 1280; default md; sections; design V3-Modal-FuelAssignment</t>
+        </is>
+      </c>
+      <c r="H224" s="3" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="I224" s="3" t="inlineStr">
+        <is>
+          <t>443.295</t>
+        </is>
+      </c>
+      <c r="J224" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K224" s="3" t="inlineStr">
+        <is>
+          <t>design PR #27439</t>
+        </is>
+      </c>
+      <c r="L224" s="3" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="3" t="n">
+        <v>223</v>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>E · Data / engine root causes</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>Fuel</t>
+        </is>
+      </c>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>Fuel evidence: odometer blank, "no GPS truck" while truck parked at pump</t>
+        </is>
+      </c>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>360 of 818 fills no station coords; 713 no GPS truck; T173 parked 3:09–4:05 PM odo 438,489.5</t>
+        </is>
+      </c>
+      <c r="F225" s="3" t="inlineStr">
+        <is>
+          <t>station never geocoded; resolver needs breadcrumb at fill minute</t>
+        </is>
+      </c>
+      <c r="G225" s="3" t="inlineStr">
+        <is>
+          <t>geocode stations; parked-hold resolver; odometer at fill</t>
+        </is>
+      </c>
+      <c r="H225" s="3" t="inlineStr">
+        <is>
+          <t>CC-2</t>
+        </is>
+      </c>
+      <c r="I225" s="3" t="inlineStr">
+        <is>
+          <t>443.296</t>
+        </is>
+      </c>
+      <c r="J225" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K225" s="3" t="inlineStr"/>
+      <c r="L225" s="3" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="3" t="n">
+        <v>224</v>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D226" s="3" t="inlineStr">
+        <is>
+          <t>CODE-COMPLETE MODE: code every row, verify at the end</t>
+        </is>
+      </c>
+      <c r="E226" s="3" t="inlineStr">
+        <is>
+          <t>owner 9:40 PM</t>
+        </is>
+      </c>
+      <c r="F226" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G226" s="3" t="inlineStr">
+        <is>
+          <t>rows assigned by seat; deadline 10-24 10:00 AM CT</t>
+        </is>
+      </c>
+      <c r="H226" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="I226" s="3" t="inlineStr">
+        <is>
+          <t>443.297</t>
+        </is>
+      </c>
+      <c r="J226" s="7" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K226" s="3" t="inlineStr">
+        <is>
+          <t>box in docs/bus/lead/boxes/2026-10-23</t>
+        </is>
+      </c>
+      <c r="L226" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:L201"/>

</xml_diff>

<commit_message>
FINDING: N/A LANE: NON-FINANCIAL — LEAD 443.297: code-complete mode — register seats reassigned (CC-1 38, CC-2 25, CC-3 22, Cursor 77, Codex 27), rows 222-224, and all 10-23 coder boxes (#27443)
Docs only: docs/bus/lead/LEAD-PENDING-REGISTER.xlsx/.md + docs/bus/lead/boxes/2026-10-23/ (40 coder instruction boxes).


Claude-Session: https://claude.ai/code/session_0112DqKNUusL2t72oep2o5Jj

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
+++ b/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L223"/>
+  <dimension ref="A1:L226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -502,7 +502,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 9:20 PM CT · every item numbered · DONE only with live proof</t>
+          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 10:15 PM CT · CODE-COMPLETE MODE (owner 9:40 PM) · deadline 10-24 10:00 AM CT</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>LEAD/CC-3</t>
+          <t>LEAD</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>CC-2 + CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>CURSOR/CC-1</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>CC-3/CURSOR</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>CURSOR/CODEX/CC-3</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>CURSOR + CC-1</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>CODEX (guard) + CURSOR (pages)</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -2948,7 +2948,7 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
@@ -3288,7 +3288,7 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
@@ -3516,7 +3516,7 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -4116,7 +4116,7 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -4376,7 +4376,7 @@
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>CURSOR (UI) + CC-1 (report APIs)</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>CC-2 + OWNER</t>
+          <t>CC-2</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>CC-2 + OWNER</t>
+          <t>CC-2</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>CC-2 + OWNER</t>
+          <t>CC-2</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>CC-2</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I100" s="3" t="inlineStr">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>CC-2</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I102" s="3" t="inlineStr">
@@ -6132,7 +6132,7 @@
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I104" s="3" t="inlineStr">
@@ -6188,7 +6188,7 @@
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I105" s="3" t="inlineStr">
@@ -6472,7 +6472,7 @@
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
-          <t>CC-3</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I110" s="3" t="inlineStr">
@@ -6584,7 +6584,7 @@
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>CODEX/CC-3</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I112" s="3" t="inlineStr">
@@ -6640,7 +6640,7 @@
       </c>
       <c r="H113" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I113" s="3" t="inlineStr">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
-          <t>CC-2</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I114" s="3" t="inlineStr">
@@ -6800,7 +6800,7 @@
       <c r="G116" s="3" t="inlineStr"/>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>CURSOR</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I116" s="3" t="inlineStr">
@@ -6844,7 +6844,7 @@
       <c r="G117" s="3" t="inlineStr"/>
       <c r="H117" s="3" t="inlineStr">
         <is>
-          <t>CC-2/CC-3</t>
+          <t>CC-2</t>
         </is>
       </c>
       <c r="I117" s="3" t="inlineStr">
@@ -6984,7 +6984,7 @@
       <c r="G120" s="3" t="inlineStr"/>
       <c r="H120" s="3" t="inlineStr">
         <is>
-          <t>CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I120" s="3" t="inlineStr">
@@ -7028,7 +7028,7 @@
       <c r="G121" s="3" t="inlineStr"/>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I121" s="3" t="inlineStr">
@@ -7204,7 +7204,7 @@
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -7384,7 +7384,7 @@
       </c>
       <c r="H127" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I127" s="3" t="inlineStr">
@@ -8344,7 +8344,7 @@
       </c>
       <c r="H143" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I143" s="3" t="inlineStr">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H147" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I147" s="3" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="H148" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I148" s="3" t="inlineStr">
@@ -8884,7 +8884,7 @@
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I152" s="3" t="inlineStr">
@@ -9004,7 +9004,7 @@
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="H155" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I155" s="3" t="inlineStr">
@@ -9124,7 +9124,7 @@
       </c>
       <c r="H156" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I156" s="3" t="inlineStr">
@@ -9184,7 +9184,7 @@
       </c>
       <c r="H157" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I157" s="3" t="inlineStr">
@@ -9244,7 +9244,7 @@
       </c>
       <c r="H158" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I158" s="3" t="inlineStr">
@@ -9304,7 +9304,7 @@
       </c>
       <c r="H159" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I159" s="3" t="inlineStr">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="H160" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I160" s="3" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="H161" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I161" s="3" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="H165" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I165" s="3" t="inlineStr">
@@ -9784,7 +9784,7 @@
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -9844,7 +9844,7 @@
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
@@ -9904,7 +9904,7 @@
       </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I169" s="3" t="inlineStr">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I170" s="3" t="inlineStr">
@@ -10204,7 +10204,7 @@
       </c>
       <c r="H174" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I174" s="3" t="inlineStr">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I175" s="3" t="inlineStr">
@@ -10324,7 +10324,7 @@
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I176" s="3" t="inlineStr">
@@ -10444,7 +10444,7 @@
       </c>
       <c r="H178" s="3" t="inlineStr">
         <is>
-          <t>CC-1 / Cursor</t>
+          <t>CC-1</t>
         </is>
       </c>
       <c r="I178" s="3" t="inlineStr">
@@ -10804,7 +10804,7 @@
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I184" s="3" t="inlineStr">
@@ -11464,7 +11464,7 @@
       </c>
       <c r="H195" s="3" t="inlineStr">
         <is>
-          <t>Lead assigns</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I195" s="3" t="inlineStr">
@@ -11704,7 +11704,7 @@
       </c>
       <c r="H199" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I199" s="3" t="inlineStr">
@@ -11764,7 +11764,7 @@
       </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>CC-3</t>
         </is>
       </c>
       <c r="I200" s="3" t="inlineStr">
@@ -11820,7 +11820,7 @@
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
-          <t>CODEX</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="I201" s="3" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>CC-2/CC-3</t>
+          <t>CC-2</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -12055,7 +12055,7 @@
       </c>
       <c r="K205" s="3" t="inlineStr">
         <is>
-          <t>AUTH-454 COMMITTED on prod (5 headers, TB 0, 7091=7091); AUTH-453 running on prod (owner OK 8:42 PM); fork: uncapped guard exit 0</t>
+          <t>AUTH-454 COMMITTED prod (TB 0); AUTH-453 150/241 on prod 10:15 PM, TB 0, retry loop (lock contention)</t>
         </is>
       </c>
       <c r="L205" s="3" t="n"/>
@@ -12372,7 +12372,7 @@
       </c>
       <c r="H211" s="3" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>Cursor</t>
         </is>
       </c>
       <c r="I211" s="3" t="inlineStr">
@@ -13023,6 +13023,170 @@
       </c>
       <c r="K223" s="3" t="inlineStr"/>
       <c r="L223" s="3" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="3" t="n">
+        <v>222</v>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="inlineStr">
+        <is>
+          <t>All modules</t>
+        </is>
+      </c>
+      <c r="D224" s="3" t="inlineStr">
+        <is>
+          <t>Popup standard app-wide + Fuel assignment popup redesign</t>
+        </is>
+      </c>
+      <c r="E224" s="3" t="inlineStr">
+        <is>
+          <t>Modal falls back to 85% width; 140 of 155 popup files pass no size</t>
+        </is>
+      </c>
+      <c r="F224" s="3" t="inlineStr">
+        <is>
+          <t>no width caps except xl</t>
+        </is>
+      </c>
+      <c r="G224" s="3" t="inlineStr">
+        <is>
+          <t>sm 480/md 720/lg 960/xl 1280; default md; sections; design V3-Modal-FuelAssignment</t>
+        </is>
+      </c>
+      <c r="H224" s="3" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="I224" s="3" t="inlineStr">
+        <is>
+          <t>443.295</t>
+        </is>
+      </c>
+      <c r="J224" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K224" s="3" t="inlineStr">
+        <is>
+          <t>design PR #27439</t>
+        </is>
+      </c>
+      <c r="L224" s="3" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="3" t="n">
+        <v>223</v>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>E · Data / engine root causes</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>Fuel</t>
+        </is>
+      </c>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>Fuel evidence: odometer blank, "no GPS truck" while truck parked at pump</t>
+        </is>
+      </c>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>360 of 818 fills no station coords; 713 no GPS truck; T173 parked 3:09–4:05 PM odo 438,489.5</t>
+        </is>
+      </c>
+      <c r="F225" s="3" t="inlineStr">
+        <is>
+          <t>station never geocoded; resolver needs breadcrumb at fill minute</t>
+        </is>
+      </c>
+      <c r="G225" s="3" t="inlineStr">
+        <is>
+          <t>geocode stations; parked-hold resolver; odometer at fill</t>
+        </is>
+      </c>
+      <c r="H225" s="3" t="inlineStr">
+        <is>
+          <t>CC-2</t>
+        </is>
+      </c>
+      <c r="I225" s="3" t="inlineStr">
+        <is>
+          <t>443.296</t>
+        </is>
+      </c>
+      <c r="J225" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K225" s="3" t="inlineStr"/>
+      <c r="L225" s="3" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="3" t="n">
+        <v>224</v>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>A · Owner requests (last 24 h)</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D226" s="3" t="inlineStr">
+        <is>
+          <t>CODE-COMPLETE MODE: code every row, verify at the end</t>
+        </is>
+      </c>
+      <c r="E226" s="3" t="inlineStr">
+        <is>
+          <t>owner 9:40 PM</t>
+        </is>
+      </c>
+      <c r="F226" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G226" s="3" t="inlineStr">
+        <is>
+          <t>rows assigned by seat; deadline 10-24 10:00 AM CT</t>
+        </is>
+      </c>
+      <c r="H226" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="I226" s="3" t="inlineStr">
+        <is>
+          <t>443.297</t>
+        </is>
+      </c>
+      <c r="J226" s="7" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K226" s="3" t="inlineStr">
+        <is>
+          <t>box in docs/bus/lead/boxes/2026-10-23</t>
+        </is>
+      </c>
+      <c r="L226" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:L201"/>

</xml_diff>

<commit_message>
FINDING: N/A LANE: NON-FINANCIAL — LEAD register 11:10 PM CT: rows 31-35, 98, 200, 211 CODED; 203 PAUSED
Docs only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0112DqKNUusL2t72oep2o5Jj
</commit_message>
<xml_diff>
--- a/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
+++ b/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
@@ -502,7 +502,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 10:15 PM CT · CODE-COMPLETE MODE (owner 9:40 PM) · deadline 10-24 10:00 AM CT</t>
+          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 11:10 PM CT · CODE-COMPLETE MODE · deadline 10-24 10:00 AM CT</t>
         </is>
       </c>
     </row>
@@ -2202,10 +2202,14 @@
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="K33" s="3" t="inlineStr"/>
+          <t>CODED</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>#27453 (Home unchanged = board)</t>
+        </is>
+      </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> 10-24 02:00 UTC</t>
@@ -2254,10 +2258,14 @@
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr"/>
+          <t>CODED</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>#27453</t>
+        </is>
+      </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> 10-24 02:00 UTC</t>
@@ -2306,10 +2314,14 @@
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="K35" s="3" t="inlineStr"/>
+          <t>CODED</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>#27453 AvP board restored</t>
+        </is>
+      </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> 10-24 02:00 UTC</t>
@@ -2362,10 +2374,14 @@
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="K36" s="3" t="inlineStr"/>
+          <t>CODED</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>#27453</t>
+        </is>
+      </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> 10-24 02:00 UTC</t>
@@ -2418,10 +2434,14 @@
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="K37" s="3" t="inlineStr"/>
+          <t>CODED</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>#27453 Manual board + opening cash</t>
+        </is>
+      </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> 10-24 02:00 UTC</t>
@@ -5918,10 +5938,14 @@
       </c>
       <c r="J100" s="7" t="inlineStr">
         <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="K100" s="3" t="inlineStr"/>
+          <t>CODED</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr">
+        <is>
+          <t>CC-1 7349992008 formatting; True-cost denominator with CC-1</t>
+        </is>
+      </c>
       <c r="L100" s="3" t="inlineStr">
         <is>
           <t>10-24 02:00 UTC</t>
@@ -11886,12 +11910,12 @@
       </c>
       <c r="J202" s="7" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>CODED</t>
         </is>
       </c>
       <c r="K202" s="3" t="inlineStr">
         <is>
-          <t>9ef89188 test 3/3, be tsc 0; push waits on main reds</t>
+          <t>#27452 eef79722</t>
         </is>
       </c>
       <c r="L202" s="3" t="n"/>
@@ -12050,12 +12074,12 @@
       </c>
       <c r="J205" s="7" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>PAUSED</t>
         </is>
       </c>
       <c r="K205" s="3" t="inlineStr">
         <is>
-          <t>AUTH-454 COMMITTED prod (TB 0); AUTH-453 150/241 on prod 10:15 PM, TB 0, retry loop (lock contention)</t>
+          <t>AUTH-454 done; AUTH-453 198/241 on prod — owner: resume after all rows coded</t>
         </is>
       </c>
       <c r="L205" s="3" t="n"/>
@@ -12494,12 +12518,12 @@
       </c>
       <c r="J213" s="7" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>CODED</t>
         </is>
       </c>
       <c r="K213" s="3" t="inlineStr">
         <is>
-          <t>162429bd guards + 7/7 tests; push after linkage green</t>
+          <t>#27453 d86e35ce</t>
         </is>
       </c>
       <c r="L213" s="3" t="n"/>

</xml_diff>

<commit_message>
FINDING: N/A LANE: NON-FINANCIAL — LEAD register 11:10 PM CT: rows 31-35, 98, 200, 211 CODED; 203 PAUSED (#27454)
Docs only.


Claude-Session: https://claude.ai/code/session_0112DqKNUusL2t72oep2o5Jj

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
+++ b/docs/bus/lead/LEAD-PENDING-REGISTER.xlsx
@@ -502,7 +502,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 10:15 PM CT · CODE-COMPLETE MODE (owner 9:40 PM) · deadline 10-24 10:00 AM CT</t>
+          <t>IH35-TMS · USMCA · LEAD PENDING REGISTER · updated 10-23-2026 11:10 PM CT · CODE-COMPLETE MODE · deadline 10-24 10:00 AM CT</t>
         </is>
       </c>
     </row>
@@ -2202,10 +2202,14 @@
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="K33" s="3" t="inlineStr"/>
+          <t>CODED</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>#27453 (Home unchanged = board)</t>
+        </is>
+      </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> 10-24 02:00 UTC</t>
@@ -2254,10 +2258,14 @@
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr"/>
+          <t>CODED</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>#27453</t>
+        </is>
+      </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> 10-24 02:00 UTC</t>
@@ -2306,10 +2314,14 @@
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="K35" s="3" t="inlineStr"/>
+          <t>CODED</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>#27453 AvP board restored</t>
+        </is>
+      </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> 10-24 02:00 UTC</t>
@@ -2362,10 +2374,14 @@
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="K36" s="3" t="inlineStr"/>
+          <t>CODED</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>#27453</t>
+        </is>
+      </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> 10-24 02:00 UTC</t>
@@ -2418,10 +2434,14 @@
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="K37" s="3" t="inlineStr"/>
+          <t>CODED</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>#27453 Manual board + opening cash</t>
+        </is>
+      </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> 10-24 02:00 UTC</t>
@@ -5918,10 +5938,14 @@
       </c>
       <c r="J100" s="7" t="inlineStr">
         <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="K100" s="3" t="inlineStr"/>
+          <t>CODED</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr">
+        <is>
+          <t>CC-1 7349992008 formatting; True-cost denominator with CC-1</t>
+        </is>
+      </c>
       <c r="L100" s="3" t="inlineStr">
         <is>
           <t>10-24 02:00 UTC</t>
@@ -11886,12 +11910,12 @@
       </c>
       <c r="J202" s="7" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>CODED</t>
         </is>
       </c>
       <c r="K202" s="3" t="inlineStr">
         <is>
-          <t>9ef89188 test 3/3, be tsc 0; push waits on main reds</t>
+          <t>#27452 eef79722</t>
         </is>
       </c>
       <c r="L202" s="3" t="n"/>
@@ -12050,12 +12074,12 @@
       </c>
       <c r="J205" s="7" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>PAUSED</t>
         </is>
       </c>
       <c r="K205" s="3" t="inlineStr">
         <is>
-          <t>AUTH-454 COMMITTED prod (TB 0); AUTH-453 150/241 on prod 10:15 PM, TB 0, retry loop (lock contention)</t>
+          <t>AUTH-454 done; AUTH-453 198/241 on prod — owner: resume after all rows coded</t>
         </is>
       </c>
       <c r="L205" s="3" t="n"/>
@@ -12494,12 +12518,12 @@
       </c>
       <c r="J213" s="7" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>CODED</t>
         </is>
       </c>
       <c r="K213" s="3" t="inlineStr">
         <is>
-          <t>162429bd guards + 7/7 tests; push after linkage green</t>
+          <t>#27453 d86e35ce</t>
         </is>
       </c>
       <c r="L213" s="3" t="n"/>

</xml_diff>